<commit_message>
Fix transcription errors in 교사별 시간표 vs 전체 교사 시간표
Cross-checked all 782 cells between the per-teacher block sheet
(used for parsing) and the master matrix sheet, found 19 mismatches
from manual transcription mistakes:
- 정우영: move-class tags (A/B) dropped from 법과사회 at 6 slots
- 김규리: Wednesday art classes off by one period
- 최승희: Friday 창체 duty missing entirely
- 이상민: 일본어회화 truncated to 일본어회 (display only)

Also fixes the earlier '1-1.' class-name typo (김규리 수5, 1-1 vs 1-1.).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RRUtttDYzF1999tCrxwK9V
</commit_message>
<xml_diff>
--- a/2026학년도_2학기_시간표(교과매핑추가).xlsx
+++ b/2026학년도_2학기_시간표(교과매핑추가).xlsx
@@ -14109,7 +14109,7 @@
       </c>
       <c r="C202" s="35" t="inlineStr">
         <is>
-          <t>법과사회</t>
+          <t>법과사회B</t>
         </is>
       </c>
       <c r="D202" s="35" t="n"/>
@@ -14146,7 +14146,7 @@
       </c>
       <c r="B204" s="58" t="inlineStr">
         <is>
-          <t>법과사회</t>
+          <t>법과사회A</t>
         </is>
       </c>
       <c r="C204" s="34" t="n"/>
@@ -14158,7 +14158,7 @@
       <c r="E204" s="34" t="n"/>
       <c r="F204" s="59" t="inlineStr">
         <is>
-          <t>법과사회</t>
+          <t>법과사회B</t>
         </is>
       </c>
     </row>
@@ -14283,13 +14283,13 @@
       </c>
       <c r="C212" s="34" t="inlineStr">
         <is>
-          <t>법과사회</t>
+          <t>법과사회A</t>
         </is>
       </c>
       <c r="D212" s="34" t="n"/>
       <c r="E212" s="34" t="inlineStr">
         <is>
-          <t>법과사회</t>
+          <t>법과사회A</t>
         </is>
       </c>
       <c r="F212" s="59" t="inlineStr">
@@ -14331,7 +14331,7 @@
       <c r="D214" s="34" t="n"/>
       <c r="E214" s="34" t="inlineStr">
         <is>
-          <t>법과사회</t>
+          <t>법과사회B</t>
         </is>
       </c>
       <c r="F214" s="59" t="n"/>
@@ -16060,7 +16060,11 @@
       </c>
       <c r="B316" s="58" t="n"/>
       <c r="C316" s="34" t="n"/>
-      <c r="D316" s="34" t="n"/>
+      <c r="D316" s="34" t="inlineStr">
+        <is>
+          <t>미술창작</t>
+        </is>
+      </c>
       <c r="E316" s="34" t="n"/>
       <c r="F316" s="59" t="n"/>
     </row>
@@ -16068,7 +16072,11 @@
       <c r="A317" s="168" t="n"/>
       <c r="B317" s="55" t="n"/>
       <c r="C317" s="56" t="n"/>
-      <c r="D317" s="56" t="n"/>
+      <c r="D317" s="56" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
       <c r="E317" s="56" t="n"/>
       <c r="F317" s="57" t="n"/>
     </row>
@@ -16104,7 +16112,7 @@
       <c r="C319" s="56" t="n"/>
       <c r="D319" s="56" t="inlineStr">
         <is>
-          <t>1-1.</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="E319" s="56" t="n"/>
@@ -16120,11 +16128,7 @@
         </is>
       </c>
       <c r="C320" s="34" t="n"/>
-      <c r="D320" s="34" t="inlineStr">
-        <is>
-          <t>미술창작</t>
-        </is>
-      </c>
+      <c r="D320" s="34" t="n"/>
       <c r="E320" s="34" t="n"/>
       <c r="F320" s="59" t="inlineStr">
         <is>
@@ -16140,11 +16144,7 @@
         </is>
       </c>
       <c r="C321" s="56" t="n"/>
-      <c r="D321" s="56" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
+      <c r="D321" s="56" t="n"/>
       <c r="E321" s="56" t="n"/>
       <c r="F321" s="57" t="n"/>
     </row>
@@ -16562,7 +16562,11 @@
       <c r="C354" s="34" t="n"/>
       <c r="D354" s="34" t="n"/>
       <c r="E354" s="34" t="n"/>
-      <c r="F354" s="59" t="n"/>
+      <c r="F354" s="59" t="inlineStr">
+        <is>
+          <t>창체</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="168" t="n"/>
@@ -16580,7 +16584,11 @@
       <c r="C356" s="34" t="n"/>
       <c r="D356" s="34" t="n"/>
       <c r="E356" s="34" t="n"/>
-      <c r="F356" s="59" t="n"/>
+      <c r="F356" s="59" t="inlineStr">
+        <is>
+          <t>창체</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="168" t="n"/>
@@ -17186,17 +17194,17 @@
       <c r="B402" s="58" t="n"/>
       <c r="C402" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="D402" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="E402" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="F402" s="59" t="n"/>
@@ -17228,17 +17236,17 @@
       <c r="B404" s="58" t="n"/>
       <c r="C404" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="D404" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="E404" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="F404" s="59" t="n"/>
@@ -17270,17 +17278,17 @@
       <c r="B406" s="58" t="n"/>
       <c r="C406" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="D406" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="E406" s="34" t="inlineStr">
         <is>
-          <t>일본어회</t>
+          <t>일본어회화</t>
         </is>
       </c>
       <c r="F406" s="59" t="n"/>

</xml_diff>

<commit_message>
Mark 수요일 6·7교시 as 공강 for every teacher, not just 9
Only 9 of 23 teachers had an explicit 공강 entry at Wednesday
periods 6-7 (both in 교사별 시간표 and the 전체 교사 시간표 matrix —
they agreed with each other, so not a transcription error, just
never filled in for teachers who never had anything scheduled
there). Added explicit 공강 for the remaining 14 teachers in both
sheets of both workbooks, so the grid now shows it consistently for
everyone, the same way 금요일 5·6교시 already shows 창체 for all 23.
No matching-logic change — 공강 already behaves identically to a
blank slot for swap/substitute purposes, this is a display/data
consistency fix.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RRUtttDYzF1999tCrxwK9V
</commit_message>
<xml_diff>
--- a/2026학년도_2학기_시간표(교과매핑추가).xlsx
+++ b/2026학년도_2학기_시간표(교과매핑추가).xlsx
@@ -2623,8 +2623,16 @@
         </is>
       </c>
       <c r="U9" s="139" t="n"/>
-      <c r="V9" s="139" t="n"/>
-      <c r="W9" s="141" t="n"/>
+      <c r="V9" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W9" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X9" s="143" t="inlineStr">
         <is>
           <t>화작</t>
@@ -2851,8 +2859,16 @@
           <t>영미</t>
         </is>
       </c>
-      <c r="V11" s="139" t="n"/>
-      <c r="W11" s="141" t="n"/>
+      <c r="V11" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W11" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X11" s="143" t="n"/>
       <c r="Y11" s="139" t="n"/>
       <c r="Z11" s="139" t="inlineStr">
@@ -4171,8 +4187,16 @@
           <t>한국사2</t>
         </is>
       </c>
-      <c r="V23" s="139" t="n"/>
-      <c r="W23" s="141" t="n"/>
+      <c r="V23" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W23" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X23" s="143" t="n"/>
       <c r="Y23" s="139" t="inlineStr">
         <is>
@@ -4399,8 +4423,16 @@
         </is>
       </c>
       <c r="U25" s="139" t="n"/>
-      <c r="V25" s="139" t="n"/>
-      <c r="W25" s="141" t="n"/>
+      <c r="V25" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W25" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X25" s="143" t="n"/>
       <c r="Y25" s="139" t="n"/>
       <c r="Z25" s="139" t="inlineStr">
@@ -4630,8 +4662,16 @@
           <t>사문탐</t>
         </is>
       </c>
-      <c r="V27" s="139" t="n"/>
-      <c r="W27" s="141" t="n"/>
+      <c r="V27" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W27" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X27" s="143" t="inlineStr">
         <is>
           <t>통사</t>
@@ -5077,8 +5117,16 @@
           <t>과탐실2</t>
         </is>
       </c>
-      <c r="V31" s="139" t="n"/>
-      <c r="W31" s="141" t="n"/>
+      <c r="V31" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W31" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X31" s="143" t="n"/>
       <c r="Y31" s="139" t="inlineStr">
         <is>
@@ -5525,8 +5573,16 @@
           <t>지구과학</t>
         </is>
       </c>
-      <c r="V35" s="139" t="n"/>
-      <c r="W35" s="141" t="n"/>
+      <c r="V35" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W35" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X35" s="143" t="inlineStr">
         <is>
           <t>환경</t>
@@ -5753,8 +5809,16 @@
           <t>스포츠</t>
         </is>
       </c>
-      <c r="V37" s="139" t="n"/>
-      <c r="W37" s="141" t="n"/>
+      <c r="V37" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W37" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X37" s="143" t="n"/>
       <c r="Y37" s="139" t="inlineStr">
         <is>
@@ -5981,8 +6045,16 @@
           <t>미술창작</t>
         </is>
       </c>
-      <c r="V39" s="139" t="n"/>
-      <c r="W39" s="141" t="n"/>
+      <c r="V39" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W39" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X39" s="143" t="n"/>
       <c r="Y39" s="139" t="n"/>
       <c r="Z39" s="139" t="n"/>
@@ -6147,8 +6219,16 @@
       </c>
       <c r="T41" s="139" t="n"/>
       <c r="U41" s="139" t="n"/>
-      <c r="V41" s="139" t="n"/>
-      <c r="W41" s="141" t="n"/>
+      <c r="V41" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W41" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X41" s="143" t="n"/>
       <c r="Y41" s="139" t="n"/>
       <c r="Z41" s="139" t="n"/>
@@ -6277,8 +6357,16 @@
         </is>
       </c>
       <c r="U43" s="139" t="n"/>
-      <c r="V43" s="139" t="n"/>
-      <c r="W43" s="141" t="n"/>
+      <c r="V43" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W43" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X43" s="143" t="n"/>
       <c r="Y43" s="139" t="n"/>
       <c r="Z43" s="139" t="n"/>
@@ -6441,8 +6529,16 @@
       </c>
       <c r="T45" s="139" t="n"/>
       <c r="U45" s="139" t="n"/>
-      <c r="V45" s="139" t="n"/>
-      <c r="W45" s="141" t="n"/>
+      <c r="V45" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W45" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X45" s="143" t="inlineStr">
         <is>
           <t>진로</t>
@@ -6609,8 +6705,16 @@
           <t>보건</t>
         </is>
       </c>
-      <c r="V47" s="139" t="n"/>
-      <c r="W47" s="141" t="n"/>
+      <c r="V47" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W47" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X47" s="143" t="n"/>
       <c r="Y47" s="139" t="n"/>
       <c r="Z47" s="139" t="n"/>
@@ -6775,8 +6879,16 @@
         </is>
       </c>
       <c r="U49" s="139" t="n"/>
-      <c r="V49" s="139" t="n"/>
-      <c r="W49" s="141" t="n"/>
+      <c r="V49" s="139" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
+      <c r="W49" s="141" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="X49" s="143" t="n"/>
       <c r="Y49" s="62" t="inlineStr">
         <is>
@@ -11557,7 +11669,11 @@
           <t>화작</t>
         </is>
       </c>
-      <c r="D50" s="34" t="n"/>
+      <c r="D50" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E50" s="34" t="n"/>
       <c r="F50" s="59" t="inlineStr">
         <is>
@@ -11587,7 +11703,11 @@
         </is>
       </c>
       <c r="C52" s="34" t="n"/>
-      <c r="D52" s="34" t="n"/>
+      <c r="D52" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E52" s="34" t="inlineStr">
         <is>
           <t>화작</t>
@@ -11870,7 +11990,11 @@
           <t>영미</t>
         </is>
       </c>
-      <c r="D68" s="34" t="n"/>
+      <c r="D68" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E68" s="34" t="n"/>
       <c r="F68" s="59" t="inlineStr">
         <is>
@@ -11900,7 +12024,11 @@
       </c>
       <c r="B70" s="58" t="n"/>
       <c r="C70" s="34" t="n"/>
-      <c r="D70" s="34" t="n"/>
+      <c r="D70" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E70" s="34" t="inlineStr">
         <is>
           <t>영미</t>
@@ -13672,7 +13800,11 @@
           <t>세계사A</t>
         </is>
       </c>
-      <c r="D176" s="34" t="n"/>
+      <c r="D176" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E176" s="34" t="inlineStr">
         <is>
           <t>세계사A</t>
@@ -13710,7 +13842,11 @@
         </is>
       </c>
       <c r="C178" s="34" t="n"/>
-      <c r="D178" s="34" t="n"/>
+      <c r="D178" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E178" s="34" t="inlineStr">
         <is>
           <t>세계사B</t>
@@ -13981,7 +14117,11 @@
           <t>통사2</t>
         </is>
       </c>
-      <c r="D194" s="34" t="n"/>
+      <c r="D194" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E194" s="34" t="inlineStr">
         <is>
           <t>생윤</t>
@@ -14019,7 +14159,11 @@
         </is>
       </c>
       <c r="C196" s="34" t="n"/>
-      <c r="D196" s="34" t="n"/>
+      <c r="D196" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E196" s="34" t="inlineStr">
         <is>
           <t>통사2</t>
@@ -14286,7 +14430,11 @@
           <t>법과사회A</t>
         </is>
       </c>
-      <c r="D212" s="34" t="n"/>
+      <c r="D212" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E212" s="34" t="inlineStr">
         <is>
           <t>법과사회A</t>
@@ -14328,7 +14476,11 @@
           <t>사문탐</t>
         </is>
       </c>
-      <c r="D214" s="34" t="n"/>
+      <c r="D214" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E214" s="34" t="inlineStr">
         <is>
           <t>법과사회B</t>
@@ -14896,7 +15048,11 @@
           <t>화학A</t>
         </is>
       </c>
-      <c r="D248" s="34" t="n"/>
+      <c r="D248" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E248" s="34" t="inlineStr">
         <is>
           <t>화학A</t>
@@ -14938,7 +15094,11 @@
           <t>진로</t>
         </is>
       </c>
-      <c r="D250" s="34" t="n"/>
+      <c r="D250" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E250" s="34" t="inlineStr">
         <is>
           <t>화학B</t>
@@ -15518,7 +15678,11 @@
         </is>
       </c>
       <c r="C284" s="34" t="n"/>
-      <c r="D284" s="34" t="n"/>
+      <c r="D284" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E284" s="34" t="inlineStr">
         <is>
           <t>환경</t>
@@ -15552,7 +15716,11 @@
       </c>
       <c r="B286" s="58" t="n"/>
       <c r="C286" s="34" t="n"/>
-      <c r="D286" s="34" t="n"/>
+      <c r="D286" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E286" s="34" t="inlineStr">
         <is>
           <t>환경</t>
@@ -15847,7 +16015,11 @@
       </c>
       <c r="B302" s="58" t="n"/>
       <c r="C302" s="34" t="n"/>
-      <c r="D302" s="34" t="n"/>
+      <c r="D302" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E302" s="34" t="inlineStr">
         <is>
           <t>체육2</t>
@@ -15885,7 +16057,11 @@
           <t>운동</t>
         </is>
       </c>
-      <c r="D304" s="34" t="n"/>
+      <c r="D304" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E304" s="34" t="n"/>
       <c r="F304" s="59" t="n"/>
     </row>
@@ -16128,7 +16304,11 @@
         </is>
       </c>
       <c r="C320" s="34" t="n"/>
-      <c r="D320" s="34" t="n"/>
+      <c r="D320" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E320" s="34" t="n"/>
       <c r="F320" s="59" t="inlineStr">
         <is>
@@ -16154,7 +16334,11 @@
       </c>
       <c r="B322" s="58" t="n"/>
       <c r="C322" s="34" t="n"/>
-      <c r="D322" s="34" t="n"/>
+      <c r="D322" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E322" s="34" t="n"/>
       <c r="F322" s="59" t="n"/>
     </row>
@@ -16345,7 +16529,11 @@
       </c>
       <c r="B338" s="58" t="n"/>
       <c r="C338" s="34" t="n"/>
-      <c r="D338" s="34" t="n"/>
+      <c r="D338" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E338" s="34" t="n"/>
       <c r="F338" s="59" t="inlineStr">
         <is>
@@ -16367,7 +16555,11 @@
       </c>
       <c r="B340" s="58" t="n"/>
       <c r="C340" s="34" t="n"/>
-      <c r="D340" s="34" t="n"/>
+      <c r="D340" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E340" s="34" t="n"/>
       <c r="F340" s="59" t="n"/>
     </row>
@@ -16582,7 +16774,11 @@
       </c>
       <c r="B356" s="58" t="n"/>
       <c r="C356" s="34" t="n"/>
-      <c r="D356" s="34" t="n"/>
+      <c r="D356" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E356" s="34" t="n"/>
       <c r="F356" s="59" t="inlineStr">
         <is>
@@ -16604,7 +16800,11 @@
       </c>
       <c r="B358" s="58" t="n"/>
       <c r="C358" s="34" t="n"/>
-      <c r="D358" s="34" t="n"/>
+      <c r="D358" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E358" s="34" t="n"/>
       <c r="F358" s="59" t="n"/>
     </row>
@@ -16831,7 +17031,11 @@
         </is>
       </c>
       <c r="C374" s="34" t="n"/>
-      <c r="D374" s="34" t="n"/>
+      <c r="D374" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E374" s="34" t="n"/>
       <c r="F374" s="59" t="inlineStr">
         <is>
@@ -16861,7 +17065,11 @@
           <t>진로직업</t>
         </is>
       </c>
-      <c r="D376" s="34" t="n"/>
+      <c r="D376" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E376" s="34" t="n"/>
       <c r="F376" s="59" t="n"/>
     </row>
@@ -17080,7 +17288,11 @@
       </c>
       <c r="B392" s="58" t="n"/>
       <c r="C392" s="34" t="n"/>
-      <c r="D392" s="34" t="n"/>
+      <c r="D392" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E392" s="34" t="n"/>
       <c r="F392" s="59" t="inlineStr">
         <is>
@@ -17102,7 +17314,11 @@
       </c>
       <c r="B394" s="58" t="n"/>
       <c r="C394" s="34" t="n"/>
-      <c r="D394" s="34" t="n"/>
+      <c r="D394" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E394" s="34" t="n"/>
       <c r="F394" s="59" t="n"/>
     </row>
@@ -17341,7 +17557,11 @@
       </c>
       <c r="B410" s="58" t="n"/>
       <c r="C410" s="34" t="n"/>
-      <c r="D410" s="34" t="n"/>
+      <c r="D410" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E410" s="34" t="n"/>
       <c r="F410" s="59" t="inlineStr">
         <is>
@@ -17363,7 +17583,11 @@
       </c>
       <c r="B412" s="58" t="n"/>
       <c r="C412" s="34" t="n"/>
-      <c r="D412" s="34" t="n"/>
+      <c r="D412" s="34" t="inlineStr">
+        <is>
+          <t>공강</t>
+        </is>
+      </c>
       <c r="E412" s="34" t="n"/>
       <c r="F412" s="59" t="n"/>
     </row>

</xml_diff>